<commit_message>
fixed bugs for spike_count (and thus simple window finder) and partially refactored; all files re-generated
</commit_message>
<xml_diff>
--- a/src/analyses/linear_regression/AffliationFrom.xlsx
+++ b/src/analyses/linear_regression/AffliationFrom.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H92"/>
+  <dimension ref="A1:H135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,16 +477,16 @@
         <v>45195</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Channel.C_005</t>
+          <t>Channel.C_011_Unit 1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>(650.0, 800.0)</t>
+          <t>(700.0, 1000.0)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -496,11 +496,11 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>7124</t>
+          <t>69X</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0.846752744023099</v>
+        <v>0.682644939242831</v>
       </c>
     </row>
     <row r="3">
@@ -511,16 +511,16 @@
         <v>45195</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Channel.C_005</t>
+          <t>Channel.C_011_Unit 1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>(650.0, 800.0)</t>
+          <t>(700.0, 1000.0)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -530,11 +530,11 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>151J</t>
+          <t>94B</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.5206496482064071</v>
+        <v>0.4458791940146123</v>
       </c>
     </row>
     <row r="4">
@@ -545,16 +545,16 @@
         <v>45195</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Channel.C_025</t>
+          <t>Channel.C_011_Unit 1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>(650.0, 800.0)</t>
+          <t>(700.0, 1000.0)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -564,11 +564,11 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>7124</t>
+          <t>143H</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0.8693924099763306</v>
+        <v>0.8100432800101968</v>
       </c>
     </row>
     <row r="5">
@@ -579,16 +579,16 @@
         <v>45195</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Channel.C_025</t>
+          <t>Channel.C_011_Unit 1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>(650.0, 800.0)</t>
+          <t>(700.0, 1000.0)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0.3802261185799178</v>
+        <v>0.3609393189937296</v>
       </c>
     </row>
     <row r="6">
@@ -613,16 +613,16 @@
         <v>45195</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Channel.C_027</t>
+          <t>Channel.C_027_Unit 2</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>(100.0, 250.0)</t>
+          <t>(150.0, 350.0)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -632,11 +632,11 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>87J</t>
+          <t>143H</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0.2520679680473592</v>
+        <v>0.3421767808292491</v>
       </c>
     </row>
     <row r="7">
@@ -647,16 +647,16 @@
         <v>45195</v>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Channel.C_027</t>
+          <t>Channel.C_002_Unit 1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>(650.0, 800.0)</t>
+          <t>(0.0, 2000.0)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -666,11 +666,11 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>7124</t>
+          <t>72X</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>0.9415590084681379</v>
+        <v>0.3672796832832588</v>
       </c>
     </row>
     <row r="8">
@@ -678,19 +678,19 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45195</v>
+        <v>45202</v>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Channel.C_027</t>
+          <t>Channel.C_006_Unit 1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>(650.0, 800.0)</t>
+          <t>(200.0, 400.0)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -700,11 +700,11 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>110E</t>
+          <t>94B</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>0.5392650734800125</v>
+        <v>0.2977273962592326</v>
       </c>
     </row>
     <row r="9">
@@ -712,19 +712,19 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45195</v>
+        <v>45202</v>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Channel.C_027</t>
+          <t>Channel.C_006_Unit 1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>(650.0, 800.0)</t>
+          <t>(200.0, 400.0)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -734,11 +734,11 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>151J</t>
+          <t>110E</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0.4368601289998348</v>
+        <v>0.5653312142197473</v>
       </c>
     </row>
     <row r="10">
@@ -746,19 +746,19 @@
         <v>8</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45195</v>
+        <v>45202</v>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Channel.C_027_Unit 1</t>
+          <t>Channel.C_006_Unit 1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>(0.0, 300.0)</t>
+          <t>(200.0, 400.0)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -768,11 +768,11 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>94B</t>
+          <t>67G</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>0.5817645073627393</v>
+        <v>0.6031440926251912</v>
       </c>
     </row>
     <row r="11">
@@ -783,16 +783,16 @@
         <v>45202</v>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Channel.C_009</t>
+          <t>Channel.C_006_Unit 1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>(200.0, 400.0)</t>
+          <t>(2150.0, 2250.0)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -802,11 +802,11 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>72X</t>
+          <t>94B</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>0.3666124185213948</v>
+        <v>0.3982841405313975</v>
       </c>
     </row>
     <row r="12">
@@ -817,16 +817,16 @@
         <v>45202</v>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Channel.C_010</t>
+          <t>Channel.C_006_Unit 1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>(300.0, 400.0)</t>
+          <t>(2150.0, 2250.0)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -836,11 +836,11 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>7124</t>
+          <t>110E</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>0.3077173046071328</v>
+        <v>0.6375135799690836</v>
       </c>
     </row>
     <row r="13">
@@ -851,16 +851,16 @@
         <v>45202</v>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Channel.C_010</t>
+          <t>Channel.C_006_Unit 1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>(300.0, 400.0)</t>
+          <t>(2150.0, 2250.0)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -870,11 +870,11 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>110E</t>
+          <t>67G</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>0.62327118841358</v>
+        <v>0.3476950927646296</v>
       </c>
     </row>
     <row r="14">
@@ -885,16 +885,16 @@
         <v>45202</v>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Channel.C_010</t>
+          <t>Channel.C_026_Unit 1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>(300.0, 400.0)</t>
+          <t>(1900.0, 2000.0)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -904,11 +904,11 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>67G</t>
+          <t>94B</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>0.6955328408610286</v>
+        <v>0.2610255501247147</v>
       </c>
     </row>
     <row r="15">
@@ -919,11 +919,11 @@
         <v>45202</v>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Channel.C_010_Unit 2</t>
+          <t>Channel.C_013_Unit 1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -938,11 +938,11 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>94B</t>
+          <t>110E</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>0.4422130458057683</v>
+        <v>0.2889622688742634</v>
       </c>
     </row>
     <row r="16">
@@ -953,11 +953,11 @@
         <v>45202</v>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Channel.C_010_Unit 2</t>
+          <t>Channel.C_013_Unit 1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -972,11 +972,11 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>110E</t>
+          <t>67G</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>0.3709514939730286</v>
+        <v>0.795782394816556</v>
       </c>
     </row>
     <row r="17">
@@ -987,11 +987,11 @@
         <v>45202</v>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Channel.C_010_Unit 2</t>
+          <t>Channel.C_013_Unit 1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1006,11 +1006,11 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>67G</t>
+          <t>87J</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>0.6331208461851939</v>
+        <v>0.3712339906462274</v>
       </c>
     </row>
     <row r="18">
@@ -1018,19 +1018,19 @@
         <v>16</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>45209</v>
+        <v>45202</v>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Channel.C_011</t>
+          <t>Channel.C_006</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>(500.0, 600.0)</t>
+          <t>(450.0, 650.0)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1040,11 +1040,11 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>110E</t>
+          <t>67G</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>0.5499779233581139</v>
+        <v>0.2700674865930591</v>
       </c>
     </row>
     <row r="19">
@@ -1052,19 +1052,19 @@
         <v>17</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>45209</v>
+        <v>45202</v>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Channel.C_022</t>
+          <t>Channel.C_010_Unit 2</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>(350.0, 500.0)</t>
+          <t>(200.0, 650.0)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1074,11 +1074,11 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>110E</t>
+          <t>94B</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>0.7410963078118331</v>
+        <v>0.4331289697452644</v>
       </c>
     </row>
     <row r="20">
@@ -1086,19 +1086,19 @@
         <v>18</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>45209</v>
+        <v>45202</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Channel.C_022</t>
+          <t>Channel.C_010_Unit 2</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>(350.0, 500.0)</t>
+          <t>(200.0, 650.0)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>67G</t>
+          <t>110E</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>0.5272282009760745</v>
+        <v>0.3847609501898419</v>
       </c>
     </row>
     <row r="21">
@@ -1120,19 +1120,19 @@
         <v>19</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>45209</v>
+        <v>45202</v>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Channel.C_022</t>
+          <t>Channel.C_010_Unit 2</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>(350.0, 500.0)</t>
+          <t>(200.0, 650.0)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1142,11 +1142,11 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>151J</t>
+          <t>67G</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>0.2905682389533276</v>
+        <v>0.6414814793918349</v>
       </c>
     </row>
     <row r="22">
@@ -1154,19 +1154,19 @@
         <v>20</v>
       </c>
       <c r="B22" s="2" t="n">
-        <v>45209</v>
+        <v>45202</v>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Channel.C_009</t>
+          <t>Channel.C_026</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>(1550.0, 1650.0)</t>
+          <t>(1000.0, 1100.0)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1180,7 +1180,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>0.4575416790085134</v>
+        <v>0.6463495239030927</v>
       </c>
     </row>
     <row r="23">
@@ -1188,19 +1188,19 @@
         <v>21</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>45209</v>
+        <v>45202</v>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Channel.C_009</t>
+          <t>Channel.C_026</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>(1550.0, 1650.0)</t>
+          <t>(1000.0, 1100.0)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1210,11 +1210,11 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>110E</t>
+          <t>151J</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>0.8105265376455064</v>
+        <v>0.6939183671643354</v>
       </c>
     </row>
     <row r="24">
@@ -1222,19 +1222,19 @@
         <v>22</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>45209</v>
+        <v>45202</v>
       </c>
       <c r="C24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Channel.C_009</t>
+          <t>Channel.C_010_Unit 2</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>(1550.0, 1650.0)</t>
+          <t>(200.0, 600.0)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1244,11 +1244,11 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>67G</t>
+          <t>94B</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>0.6098636637370898</v>
+        <v>0.4422130458057683</v>
       </c>
     </row>
     <row r="25">
@@ -1256,19 +1256,19 @@
         <v>23</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>45209</v>
+        <v>45202</v>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Channel.C_009</t>
+          <t>Channel.C_010_Unit 2</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>(1550.0, 1650.0)</t>
+          <t>(200.0, 600.0)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1278,11 +1278,11 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>151J</t>
+          <t>110E</t>
         </is>
       </c>
       <c r="H25" t="n">
-        <v>0.2983461497945854</v>
+        <v>0.3709514939730286</v>
       </c>
     </row>
     <row r="26">
@@ -1290,19 +1290,19 @@
         <v>24</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>45210</v>
+        <v>45202</v>
       </c>
       <c r="C26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Channel.C_002</t>
+          <t>Channel.C_010_Unit 2</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>(1050.0, 1150.0)</t>
+          <t>(200.0, 600.0)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1316,7 +1316,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>0.2909000265412877</v>
+        <v>0.6331208461851939</v>
       </c>
     </row>
     <row r="27">
@@ -1324,19 +1324,19 @@
         <v>25</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>45210</v>
+        <v>45203</v>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Channel.C_022</t>
+          <t>Channel.C_004_Unit 1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>(1950.0, 2050.0)</t>
+          <t>(100.0, 700.0)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1346,11 +1346,11 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>67G</t>
+          <t>72X</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>0.328219702806321</v>
+        <v>0.318052804647826</v>
       </c>
     </row>
     <row r="28">
@@ -1358,19 +1358,19 @@
         <v>26</v>
       </c>
       <c r="B28" s="2" t="n">
-        <v>45210</v>
+        <v>45203</v>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Channel.C_002</t>
+          <t>Channel.C_019_Unit 3</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>(0.0, 2000.0)</t>
+          <t>(100.0, 500.0)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1380,11 +1380,11 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>94B</t>
+          <t>72X</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>0.8675278958776332</v>
+        <v>0.2744308083873658</v>
       </c>
     </row>
     <row r="29">
@@ -1392,14 +1392,14 @@
         <v>27</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>45210</v>
+        <v>45203</v>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Channel.C_002</t>
+          <t>Channel.C_020_Unit 2</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1414,11 +1414,11 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>143H</t>
+          <t>151J</t>
         </is>
       </c>
       <c r="H29" t="n">
-        <v>0.2696200995385124</v>
+        <v>0.2588743825630291</v>
       </c>
     </row>
     <row r="30">
@@ -1426,19 +1426,19 @@
         <v>28</v>
       </c>
       <c r="B30" s="2" t="n">
-        <v>45226</v>
+        <v>45203</v>
       </c>
       <c r="C30" t="n">
         <v>3</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Channel.C_013</t>
+          <t>Channel.C_004_Unit 2</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>(1600.0, 1700.0)</t>
+          <t>(100.0, 500.0)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1448,11 +1448,11 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>94B</t>
+          <t>7124</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>0.4178005655421696</v>
+        <v>0.6432405607155123</v>
       </c>
     </row>
     <row r="31">
@@ -1460,19 +1460,19 @@
         <v>29</v>
       </c>
       <c r="B31" s="2" t="n">
-        <v>45226</v>
+        <v>45203</v>
       </c>
       <c r="C31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Channel.C_011</t>
+          <t>Channel.C_004_Unit 2</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>(200.0, 650.0)</t>
+          <t>(100.0, 500.0)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1482,11 +1482,11 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>69X</t>
+          <t>67G</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>0.3279387704494694</v>
+        <v>0.3149062017404239</v>
       </c>
     </row>
     <row r="32">
@@ -1494,19 +1494,19 @@
         <v>30</v>
       </c>
       <c r="B32" s="2" t="n">
-        <v>45226</v>
+        <v>45203</v>
       </c>
       <c r="C32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Channel.C_011</t>
+          <t>Channel.C_009_Unit 1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>(200.0, 650.0)</t>
+          <t>(150.0, 500.0)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1516,11 +1516,11 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>72X</t>
+          <t>7124</t>
         </is>
       </c>
       <c r="H32" t="n">
-        <v>0.3290358360745368</v>
+        <v>0.3510189344741903</v>
       </c>
     </row>
     <row r="33">
@@ -1528,19 +1528,19 @@
         <v>31</v>
       </c>
       <c r="B33" s="2" t="n">
-        <v>45226</v>
+        <v>45203</v>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Channel.C_011</t>
+          <t>Channel.C_009_Unit 1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>(200.0, 650.0)</t>
+          <t>(150.0, 500.0)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1550,11 +1550,11 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>143H</t>
+          <t>110E</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>0.3816277254694441</v>
+        <v>0.3462018475808314</v>
       </c>
     </row>
     <row r="34">
@@ -1562,19 +1562,19 @@
         <v>32</v>
       </c>
       <c r="B34" s="2" t="n">
-        <v>45226</v>
+        <v>45203</v>
       </c>
       <c r="C34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Channel.C_020</t>
+          <t>Channel.C_009_Unit 1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>(200.0, 550.0)</t>
+          <t>(150.0, 500.0)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1584,11 +1584,11 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>69X</t>
+          <t>67G</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>0.3930583234219406</v>
+        <v>0.6116294559800947</v>
       </c>
     </row>
     <row r="35">
@@ -1596,19 +1596,19 @@
         <v>33</v>
       </c>
       <c r="B35" s="2" t="n">
-        <v>45226</v>
+        <v>45203</v>
       </c>
       <c r="C35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Channel.C_020</t>
+          <t>Channel.C_009_Unit 3</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>(200.0, 550.0)</t>
+          <t>(100.0, 450.0)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1618,11 +1618,11 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>72X</t>
+          <t>7124</t>
         </is>
       </c>
       <c r="H35" t="n">
-        <v>0.3779246126588073</v>
+        <v>0.6218203927665136</v>
       </c>
     </row>
     <row r="36">
@@ -1630,19 +1630,19 @@
         <v>34</v>
       </c>
       <c r="B36" s="2" t="n">
-        <v>45226</v>
+        <v>45203</v>
       </c>
       <c r="C36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Channel.C_020</t>
+          <t>Channel.C_009_Unit 3</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>(200.0, 550.0)</t>
+          <t>(100.0, 450.0)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1652,11 +1652,11 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>143H</t>
+          <t>87J</t>
         </is>
       </c>
       <c r="H36" t="n">
-        <v>0.2521787186341514</v>
+        <v>0.2618516663419962</v>
       </c>
     </row>
     <row r="37">
@@ -1664,19 +1664,19 @@
         <v>35</v>
       </c>
       <c r="B37" s="2" t="n">
-        <v>45226</v>
+        <v>45203</v>
       </c>
       <c r="C37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Channel.C_011</t>
+          <t>Channel.C_009_Unit 3</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>(0.0, 750.0)</t>
+          <t>(100.0, 450.0)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1686,11 +1686,11 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>72X</t>
+          <t>151J</t>
         </is>
       </c>
       <c r="H37" t="n">
-        <v>0.2791765997635105</v>
+        <v>0.6294724530648885</v>
       </c>
     </row>
     <row r="38">
@@ -1698,19 +1698,19 @@
         <v>36</v>
       </c>
       <c r="B38" s="2" t="n">
-        <v>45226</v>
+        <v>45203</v>
       </c>
       <c r="C38" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Channel.C_011</t>
+          <t>Channel.C_002_Unit 1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>(0.0, 750.0)</t>
+          <t>(0.0, 500.0)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1720,11 +1720,11 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>143H</t>
+          <t>67G</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>0.3465263566224303</v>
+        <v>0.2953001542920796</v>
       </c>
     </row>
     <row r="39">
@@ -1732,19 +1732,19 @@
         <v>37</v>
       </c>
       <c r="B39" s="2" t="n">
-        <v>45226</v>
+        <v>45203</v>
       </c>
       <c r="C39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Channel.C_011</t>
+          <t>Channel.C_004_Unit 2</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>(0.0, 750.0)</t>
+          <t>(0.0, 500.0)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1754,11 +1754,11 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>151J</t>
+          <t>7124</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>0.269613901140984</v>
+        <v>0.6897840156944492</v>
       </c>
     </row>
     <row r="40">
@@ -1766,19 +1766,19 @@
         <v>38</v>
       </c>
       <c r="B40" s="2" t="n">
-        <v>45226</v>
+        <v>45203</v>
       </c>
       <c r="C40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Channel.C_020</t>
+          <t>Channel.C_004_Unit 2</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>(0.0, 750.0)</t>
+          <t>(0.0, 500.0)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1788,11 +1788,11 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>69X</t>
+          <t>67G</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>0.3052313426782758</v>
+        <v>0.4471080973494221</v>
       </c>
     </row>
     <row r="41">
@@ -1800,19 +1800,19 @@
         <v>39</v>
       </c>
       <c r="B41" s="2" t="n">
-        <v>45226</v>
+        <v>45203</v>
       </c>
       <c r="C41" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Channel.C_020</t>
+          <t>Channel.C_009_Unit 1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>(0.0, 750.0)</t>
+          <t>(0.0, 2000.0)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -1822,11 +1822,11 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>72X</t>
+          <t>110E</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>0.3103121198915697</v>
+        <v>0.3375248657022238</v>
       </c>
     </row>
     <row r="42">
@@ -1834,19 +1834,19 @@
         <v>40</v>
       </c>
       <c r="B42" s="2" t="n">
-        <v>45226</v>
+        <v>45203</v>
       </c>
       <c r="C42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Channel.C_020</t>
+          <t>Channel.C_009_Unit 1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>(0.0, 750.0)</t>
+          <t>(0.0, 2000.0)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -1856,11 +1856,11 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>143H</t>
+          <t>67G</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>0.3238740985716736</v>
+        <v>0.7267094527212836</v>
       </c>
     </row>
     <row r="43">
@@ -1868,19 +1868,19 @@
         <v>41</v>
       </c>
       <c r="B43" s="2" t="n">
-        <v>45252</v>
+        <v>45203</v>
       </c>
       <c r="C43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Channel.C_011</t>
+          <t>Channel.C_009_Unit 3</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>(1900.0, 2050.0)</t>
+          <t>(0.0, 700.0)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -1890,11 +1890,11 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>94B</t>
+          <t>7124</t>
         </is>
       </c>
       <c r="H43" t="n">
-        <v>0.3071389913899139</v>
+        <v>0.4502716604271683</v>
       </c>
     </row>
     <row r="44">
@@ -1902,19 +1902,19 @@
         <v>42</v>
       </c>
       <c r="B44" s="2" t="n">
-        <v>45274</v>
+        <v>45203</v>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Channel.C_024</t>
+          <t>Channel.C_009_Unit 3</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>(1400.0, 1550.0)</t>
+          <t>(0.0, 700.0)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -1924,11 +1924,11 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>69X</t>
+          <t>94B</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>0.7034114986321064</v>
+        <v>0.3517633745988208</v>
       </c>
     </row>
     <row r="45">
@@ -1936,19 +1936,19 @@
         <v>43</v>
       </c>
       <c r="B45" s="2" t="n">
-        <v>45274</v>
+        <v>45203</v>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Channel.C_024</t>
+          <t>Channel.C_009_Unit 3</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>(1400.0, 1550.0)</t>
+          <t>(0.0, 700.0)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>143H</t>
+          <t>87J</t>
         </is>
       </c>
       <c r="H45" t="n">
-        <v>0.7375377608448062</v>
+        <v>0.3024097487640171</v>
       </c>
     </row>
     <row r="46">
@@ -1970,19 +1970,19 @@
         <v>44</v>
       </c>
       <c r="B46" s="2" t="n">
-        <v>45274</v>
+        <v>45203</v>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Channel.C_024</t>
+          <t>Channel.C_009_Unit 3</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>(1400.0, 1550.0)</t>
+          <t>(0.0, 700.0)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -1996,7 +1996,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>0.2529760373596879</v>
+        <v>0.5121339664486457</v>
       </c>
     </row>
     <row r="47">
@@ -2004,19 +2004,19 @@
         <v>45</v>
       </c>
       <c r="B47" s="2" t="n">
-        <v>45274</v>
+        <v>45203</v>
       </c>
       <c r="C47" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Channel.C_026</t>
+          <t>Channel.C_021_Unit 2</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>(750.0, 850.0)</t>
+          <t>(150.0, 450.0)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2026,11 +2026,11 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>94B</t>
+          <t>110E</t>
         </is>
       </c>
       <c r="H47" t="n">
-        <v>0.5498364483056309</v>
+        <v>0.3147223813775001</v>
       </c>
     </row>
     <row r="48">
@@ -2038,19 +2038,19 @@
         <v>46</v>
       </c>
       <c r="B48" s="2" t="n">
-        <v>45274</v>
+        <v>45203</v>
       </c>
       <c r="C48" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Channel.C_026</t>
+          <t>Channel.C_021_Unit 2</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>(750.0, 850.0)</t>
+          <t>(150.0, 450.0)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2060,11 +2060,11 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>110E</t>
+          <t>67G</t>
         </is>
       </c>
       <c r="H48" t="n">
-        <v>0.3609918944910017</v>
+        <v>0.352239170908569</v>
       </c>
     </row>
     <row r="49">
@@ -2072,19 +2072,19 @@
         <v>47</v>
       </c>
       <c r="B49" s="2" t="n">
-        <v>45274</v>
+        <v>45203</v>
       </c>
       <c r="C49" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Channel.C_026</t>
+          <t>Channel.C_022_Unit 2</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>(750.0, 850.0)</t>
+          <t>(150.0, 650.0)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2094,11 +2094,11 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>67G</t>
+          <t>69X</t>
         </is>
       </c>
       <c r="H49" t="n">
-        <v>0.3353857064569163</v>
+        <v>0.3096719110618438</v>
       </c>
     </row>
     <row r="50">
@@ -2106,19 +2106,19 @@
         <v>48</v>
       </c>
       <c r="B50" s="2" t="n">
-        <v>45274</v>
+        <v>45203</v>
       </c>
       <c r="C50" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Channel.C_026</t>
+          <t>Channel.C_022_Unit 2</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>(750.0, 850.0)</t>
+          <t>(150.0, 650.0)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2128,11 +2128,11 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>143H</t>
+          <t>72X</t>
         </is>
       </c>
       <c r="H50" t="n">
-        <v>0.2837259602768265</v>
+        <v>0.7777602544873736</v>
       </c>
     </row>
     <row r="51">
@@ -2140,19 +2140,19 @@
         <v>49</v>
       </c>
       <c r="B51" s="2" t="n">
-        <v>45278</v>
+        <v>45203</v>
       </c>
       <c r="C51" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Channel.C_029</t>
+          <t>Channel.C_022_Unit 2</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>(50.0, 150.0)</t>
+          <t>(150.0, 650.0)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2162,11 +2162,11 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>69X</t>
+          <t>87J</t>
         </is>
       </c>
       <c r="H51" t="n">
-        <v>0.6061830872600088</v>
+        <v>0.2993276162522219</v>
       </c>
     </row>
     <row r="52">
@@ -2174,19 +2174,19 @@
         <v>50</v>
       </c>
       <c r="B52" s="2" t="n">
-        <v>45278</v>
+        <v>45203</v>
       </c>
       <c r="C52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Channel.C_029</t>
+          <t>Channel.C_027_Unit 1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>(50.0, 150.0)</t>
+          <t>(350.0, 650.0)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2200,7 +2200,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>0.7093947454917098</v>
+        <v>0.3515521378633123</v>
       </c>
     </row>
     <row r="53">
@@ -2208,19 +2208,19 @@
         <v>51</v>
       </c>
       <c r="B53" s="2" t="n">
-        <v>45195</v>
+        <v>45203</v>
       </c>
       <c r="C53" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Channel.C_002_Unit 1</t>
+          <t>Channel.C_027_Unit 1</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>(0.0, 2000.0)</t>
+          <t>(350.0, 650.0)</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2230,11 +2230,11 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>72X</t>
+          <t>94B</t>
         </is>
       </c>
       <c r="H53" t="n">
-        <v>0.3672796832832588</v>
+        <v>0.4723308202422946</v>
       </c>
     </row>
     <row r="54">
@@ -2242,19 +2242,19 @@
         <v>52</v>
       </c>
       <c r="B54" s="2" t="n">
-        <v>45202</v>
+        <v>45203</v>
       </c>
       <c r="C54" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Channel.C_013_Unit 1</t>
+          <t>Channel.C_027_Unit 1</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>(200.0, 600.0)</t>
+          <t>(350.0, 650.0)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2264,11 +2264,11 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>110E</t>
+          <t>87J</t>
         </is>
       </c>
       <c r="H54" t="n">
-        <v>0.2889622688742634</v>
+        <v>0.5212394431824801</v>
       </c>
     </row>
     <row r="55">
@@ -2276,19 +2276,19 @@
         <v>53</v>
       </c>
       <c r="B55" s="2" t="n">
-        <v>45202</v>
+        <v>45203</v>
       </c>
       <c r="C55" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Channel.C_013_Unit 1</t>
+          <t>Channel.C_022_Unit 2</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>(200.0, 600.0)</t>
+          <t>(0.0, 750.0)</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2298,11 +2298,11 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>67G</t>
+          <t>69X</t>
         </is>
       </c>
       <c r="H55" t="n">
-        <v>0.795782394816556</v>
+        <v>0.2719400477093306</v>
       </c>
     </row>
     <row r="56">
@@ -2310,19 +2310,19 @@
         <v>54</v>
       </c>
       <c r="B56" s="2" t="n">
-        <v>45202</v>
+        <v>45203</v>
       </c>
       <c r="C56" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Channel.C_013_Unit 1</t>
+          <t>Channel.C_022_Unit 2</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>(200.0, 600.0)</t>
+          <t>(0.0, 750.0)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2332,11 +2332,11 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>87J</t>
+          <t>72X</t>
         </is>
       </c>
       <c r="H56" t="n">
-        <v>0.3712339906462274</v>
+        <v>0.8042173855060024</v>
       </c>
     </row>
     <row r="57">
@@ -2347,16 +2347,16 @@
         <v>45203</v>
       </c>
       <c r="C57" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Channel.C_004_Unit 1</t>
+          <t>Channel.C_022_Unit 2</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>(100.0, 700.0)</t>
+          <t>(0.0, 750.0)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2366,11 +2366,11 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>72X</t>
+          <t>87J</t>
         </is>
       </c>
       <c r="H57" t="n">
-        <v>0.318052804647826</v>
+        <v>0.3363728734178588</v>
       </c>
     </row>
     <row r="58">
@@ -2381,16 +2381,16 @@
         <v>45203</v>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Channel.C_019_Unit 3</t>
+          <t>Channel.C_027_Unit 1</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>(100.0, 500.0)</t>
+          <t>(250.0, 750.0)</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2404,7 +2404,7 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>0.2744308083873658</v>
+        <v>0.3461079436204199</v>
       </c>
     </row>
     <row r="59">
@@ -2415,16 +2415,16 @@
         <v>45203</v>
       </c>
       <c r="C59" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Channel.C_020_Unit 2</t>
+          <t>Channel.C_027_Unit 1</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>(0.0, 2000.0)</t>
+          <t>(250.0, 750.0)</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2434,11 +2434,11 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>151J</t>
+          <t>94B</t>
         </is>
       </c>
       <c r="H59" t="n">
-        <v>0.2588743825630291</v>
+        <v>0.4326329603413315</v>
       </c>
     </row>
     <row r="60">
@@ -2449,16 +2449,16 @@
         <v>45203</v>
       </c>
       <c r="C60" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Channel.C_002_Unit 1</t>
+          <t>Channel.C_027_Unit 1</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>(0.0, 500.0)</t>
+          <t>(250.0, 750.0)</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2468,11 +2468,11 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>67G</t>
+          <t>87J</t>
         </is>
       </c>
       <c r="H60" t="n">
-        <v>0.2953001542920796</v>
+        <v>0.5460127349909036</v>
       </c>
     </row>
     <row r="61">
@@ -2480,19 +2480,19 @@
         <v>59</v>
       </c>
       <c r="B61" s="2" t="n">
-        <v>45203</v>
+        <v>45204</v>
       </c>
       <c r="C61" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Channel.C_004_Unit 2</t>
+          <t>Channel.C_004_Unit 1</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>(0.0, 500.0)</t>
+          <t>(1000.0, 1100.0)</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2502,11 +2502,11 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>7124</t>
+          <t>143H</t>
         </is>
       </c>
       <c r="H61" t="n">
-        <v>0.6897840156944492</v>
+        <v>0.326512106160155</v>
       </c>
     </row>
     <row r="62">
@@ -2514,19 +2514,19 @@
         <v>60</v>
       </c>
       <c r="B62" s="2" t="n">
-        <v>45203</v>
+        <v>45204</v>
       </c>
       <c r="C62" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Channel.C_004_Unit 2</t>
+          <t>Channel.C_004_Unit 1</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>(0.0, 500.0)</t>
+          <t>(1000.0, 1100.0)</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2536,11 +2536,11 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>67G</t>
+          <t>151J</t>
         </is>
       </c>
       <c r="H62" t="n">
-        <v>0.4471080973494221</v>
+        <v>0.2910446637041499</v>
       </c>
     </row>
     <row r="63">
@@ -2548,14 +2548,14 @@
         <v>61</v>
       </c>
       <c r="B63" s="2" t="n">
-        <v>45203</v>
+        <v>45204</v>
       </c>
       <c r="C63" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Channel.C_009_Unit 1</t>
+          <t>Channel.C_004</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2570,11 +2570,11 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>110E</t>
+          <t>143H</t>
         </is>
       </c>
       <c r="H63" t="n">
-        <v>0.3375248657022238</v>
+        <v>0.5355470120987982</v>
       </c>
     </row>
     <row r="64">
@@ -2582,10 +2582,10 @@
         <v>62</v>
       </c>
       <c r="B64" s="2" t="n">
-        <v>45203</v>
+        <v>45204</v>
       </c>
       <c r="C64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -2594,7 +2594,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>(0.0, 2000.0)</t>
+          <t>(500.0, 850.0)</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -2604,11 +2604,11 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>67G</t>
+          <t>7124</t>
         </is>
       </c>
       <c r="H64" t="n">
-        <v>0.7267094527212836</v>
+        <v>0.3905221746467761</v>
       </c>
     </row>
     <row r="65">
@@ -2616,19 +2616,19 @@
         <v>63</v>
       </c>
       <c r="B65" s="2" t="n">
-        <v>45203</v>
+        <v>45204</v>
       </c>
       <c r="C65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Channel.C_009_Unit 3</t>
+          <t>Channel.C_009_Unit 1</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>(0.0, 700.0)</t>
+          <t>(500.0, 850.0)</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -2638,11 +2638,11 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>7124</t>
+          <t>110E</t>
         </is>
       </c>
       <c r="H65" t="n">
-        <v>0.4502716604271683</v>
+        <v>0.2677500524218914</v>
       </c>
     </row>
     <row r="66">
@@ -2650,19 +2650,19 @@
         <v>64</v>
       </c>
       <c r="B66" s="2" t="n">
-        <v>45203</v>
+        <v>45204</v>
       </c>
       <c r="C66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Channel.C_009_Unit 3</t>
+          <t>Channel.C_009_Unit 1</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>(0.0, 700.0)</t>
+          <t>(500.0, 850.0)</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -2672,11 +2672,11 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>94B</t>
+          <t>151J</t>
         </is>
       </c>
       <c r="H66" t="n">
-        <v>0.3517633745988208</v>
+        <v>0.3422574302405645</v>
       </c>
     </row>
     <row r="67">
@@ -2684,19 +2684,19 @@
         <v>65</v>
       </c>
       <c r="B67" s="2" t="n">
-        <v>45203</v>
+        <v>45204</v>
       </c>
       <c r="C67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Channel.C_009_Unit 3</t>
+          <t>Channel.C_019_Unit 2</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>(0.0, 700.0)</t>
+          <t>(2200.0, 2300.0)</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -2706,11 +2706,11 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>87J</t>
+          <t>94B</t>
         </is>
       </c>
       <c r="H67" t="n">
-        <v>0.3024097487640171</v>
+        <v>0.3867960657628556</v>
       </c>
     </row>
     <row r="68">
@@ -2718,19 +2718,19 @@
         <v>66</v>
       </c>
       <c r="B68" s="2" t="n">
-        <v>45203</v>
+        <v>45208</v>
       </c>
       <c r="C68" t="n">
         <v>3</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Channel.C_009_Unit 3</t>
+          <t>Channel.C_013</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>(0.0, 700.0)</t>
+          <t>(600.0, 750.0)</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -2740,11 +2740,11 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>151J</t>
+          <t>7124</t>
         </is>
       </c>
       <c r="H68" t="n">
-        <v>0.5121339664486457</v>
+        <v>0.4645989844056319</v>
       </c>
     </row>
     <row r="69">
@@ -2752,19 +2752,19 @@
         <v>67</v>
       </c>
       <c r="B69" s="2" t="n">
-        <v>45203</v>
+        <v>45208</v>
       </c>
       <c r="C69" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Channel.C_022_Unit 2</t>
+          <t>Channel.C_013</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>(0.0, 750.0)</t>
+          <t>(600.0, 750.0)</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -2774,11 +2774,11 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>69X</t>
+          <t>151J</t>
         </is>
       </c>
       <c r="H69" t="n">
-        <v>0.2719400477093306</v>
+        <v>0.4882397822645851</v>
       </c>
     </row>
     <row r="70">
@@ -2786,19 +2786,19 @@
         <v>68</v>
       </c>
       <c r="B70" s="2" t="n">
-        <v>45203</v>
+        <v>45209</v>
       </c>
       <c r="C70" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Channel.C_022_Unit 2</t>
+          <t>Channel.C_011</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>(0.0, 750.0)</t>
+          <t>(400.0, 600.0)</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -2812,7 +2812,7 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>0.8042173855060024</v>
+        <v>0.4265954031643241</v>
       </c>
     </row>
     <row r="71">
@@ -2820,19 +2820,19 @@
         <v>69</v>
       </c>
       <c r="B71" s="2" t="n">
-        <v>45203</v>
+        <v>45209</v>
       </c>
       <c r="C71" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Channel.C_022_Unit 2</t>
+          <t>Channel.C_011</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>(0.0, 750.0)</t>
+          <t>(400.0, 600.0)</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -2842,11 +2842,11 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>87J</t>
+          <t>110E</t>
         </is>
       </c>
       <c r="H71" t="n">
-        <v>0.3363728734178588</v>
+        <v>0.3397733706873844</v>
       </c>
     </row>
     <row r="72">
@@ -2854,19 +2854,19 @@
         <v>70</v>
       </c>
       <c r="B72" s="2" t="n">
-        <v>45203</v>
+        <v>45209</v>
       </c>
       <c r="C72" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Channel.C_027_Unit 1</t>
+          <t>Channel.C_011</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>(250.0, 750.0)</t>
+          <t>(400.0, 600.0)</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -2876,11 +2876,11 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>72X</t>
+          <t>87J</t>
         </is>
       </c>
       <c r="H72" t="n">
-        <v>0.3461079436204199</v>
+        <v>0.3388045713326526</v>
       </c>
     </row>
     <row r="73">
@@ -2888,19 +2888,19 @@
         <v>71</v>
       </c>
       <c r="B73" s="2" t="n">
-        <v>45203</v>
+        <v>45209</v>
       </c>
       <c r="C73" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Channel.C_027_Unit 1</t>
+          <t>Channel.C_021</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>(250.0, 750.0)</t>
+          <t>(300.0, 550.0)</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -2910,11 +2910,11 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>94B</t>
+          <t>110E</t>
         </is>
       </c>
       <c r="H73" t="n">
-        <v>0.4326329603413315</v>
+        <v>0.3536063699204142</v>
       </c>
     </row>
     <row r="74">
@@ -2922,19 +2922,19 @@
         <v>72</v>
       </c>
       <c r="B74" s="2" t="n">
-        <v>45203</v>
+        <v>45209</v>
       </c>
       <c r="C74" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Channel.C_027_Unit 1</t>
+          <t>Channel.C_021</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>(250.0, 750.0)</t>
+          <t>(300.0, 550.0)</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -2944,11 +2944,11 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>87J</t>
+          <t>67G</t>
         </is>
       </c>
       <c r="H74" t="n">
-        <v>0.5460127349909036</v>
+        <v>0.5633878722645482</v>
       </c>
     </row>
     <row r="75">
@@ -2956,19 +2956,19 @@
         <v>73</v>
       </c>
       <c r="B75" s="2" t="n">
-        <v>45204</v>
+        <v>45209</v>
       </c>
       <c r="C75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Channel.C_004</t>
+          <t>Channel.C_021</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>(0.0, 2000.0)</t>
+          <t>(300.0, 550.0)</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -2978,11 +2978,11 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>143H</t>
+          <t>87J</t>
         </is>
       </c>
       <c r="H75" t="n">
-        <v>0.5355470120987982</v>
+        <v>0.43325954095477</v>
       </c>
     </row>
     <row r="76">
@@ -2990,19 +2990,19 @@
         <v>74</v>
       </c>
       <c r="B76" s="2" t="n">
-        <v>45210</v>
+        <v>45209</v>
       </c>
       <c r="C76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Channel.C_002</t>
+          <t>Channel.C_021</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>(100.0, 500.0)</t>
+          <t>(300.0, 550.0)</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3012,11 +3012,11 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>110E</t>
+          <t>151J</t>
         </is>
       </c>
       <c r="H76" t="n">
-        <v>0.7596852354104493</v>
+        <v>0.3395775941230487</v>
       </c>
     </row>
     <row r="77">
@@ -3024,19 +3024,19 @@
         <v>75</v>
       </c>
       <c r="B77" s="2" t="n">
-        <v>45210</v>
+        <v>45209</v>
       </c>
       <c r="C77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Channel.C_002</t>
+          <t>Channel.C_021</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>(100.0, 500.0)</t>
+          <t>(1550.0, 1650.0)</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3046,11 +3046,11 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>67G</t>
+          <t>110E</t>
         </is>
       </c>
       <c r="H77" t="n">
-        <v>0.3391859365371409</v>
+        <v>0.3473383574137187</v>
       </c>
     </row>
     <row r="78">
@@ -3058,10 +3058,10 @@
         <v>76</v>
       </c>
       <c r="B78" s="2" t="n">
-        <v>45223</v>
+        <v>45210</v>
       </c>
       <c r="C78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>(250.0, 750.0)</t>
+          <t>(150.0, 400.0)</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3080,11 +3080,11 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>94B</t>
+          <t>7124</t>
         </is>
       </c>
       <c r="H78" t="n">
-        <v>0.7461224024765438</v>
+        <v>0.4533305958355019</v>
       </c>
     </row>
     <row r="79">
@@ -3092,10 +3092,10 @@
         <v>77</v>
       </c>
       <c r="B79" s="2" t="n">
-        <v>45223</v>
+        <v>45210</v>
       </c>
       <c r="C79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3104,7 +3104,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>(250.0, 750.0)</t>
+          <t>(150.0, 400.0)</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3114,11 +3114,11 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>143H</t>
+          <t>110E</t>
         </is>
       </c>
       <c r="H79" t="n">
-        <v>0.261013043787052</v>
+        <v>0.8395531510322347</v>
       </c>
     </row>
     <row r="80">
@@ -3126,10 +3126,10 @@
         <v>78</v>
       </c>
       <c r="B80" s="2" t="n">
-        <v>45223</v>
+        <v>45210</v>
       </c>
       <c r="C80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3138,7 +3138,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>(250.0, 750.0)</t>
+          <t>(150.0, 400.0)</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3148,11 +3148,11 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>151J</t>
+          <t>67G</t>
         </is>
       </c>
       <c r="H80" t="n">
-        <v>0.4522559139679887</v>
+        <v>0.4311730900701681</v>
       </c>
     </row>
     <row r="81">
@@ -3160,19 +3160,19 @@
         <v>79</v>
       </c>
       <c r="B81" s="2" t="n">
-        <v>45230</v>
+        <v>45210</v>
       </c>
       <c r="C81" t="n">
         <v>1</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Channel.C_005</t>
+          <t>Channel.C_010</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>(250.0, 600.0)</t>
+          <t>(2000.0, 2200.0)</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3182,11 +3182,11 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>7124</t>
+          <t>72X</t>
         </is>
       </c>
       <c r="H81" t="n">
-        <v>0.4626862340052377</v>
+        <v>0.45657522203673</v>
       </c>
     </row>
     <row r="82">
@@ -3194,19 +3194,19 @@
         <v>80</v>
       </c>
       <c r="B82" s="2" t="n">
-        <v>45230</v>
+        <v>45210</v>
       </c>
       <c r="C82" t="n">
         <v>1</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Channel.C_005</t>
+          <t>Channel.C_010</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>(250.0, 600.0)</t>
+          <t>(2000.0, 2200.0)</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -3216,11 +3216,11 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>143H</t>
+          <t>94B</t>
         </is>
       </c>
       <c r="H82" t="n">
-        <v>0.2784554922691393</v>
+        <v>0.5807974437545389</v>
       </c>
     </row>
     <row r="83">
@@ -3228,19 +3228,19 @@
         <v>81</v>
       </c>
       <c r="B83" s="2" t="n">
-        <v>45230</v>
+        <v>45210</v>
       </c>
       <c r="C83" t="n">
         <v>1</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Channel.C_005</t>
+          <t>Channel.C_010</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>(250.0, 600.0)</t>
+          <t>(2000.0, 2200.0)</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3254,7 +3254,7 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>0.3519294547137312</v>
+        <v>0.8620446123931468</v>
       </c>
     </row>
     <row r="84">
@@ -3262,19 +3262,19 @@
         <v>82</v>
       </c>
       <c r="B84" s="2" t="n">
-        <v>45230</v>
+        <v>45210</v>
       </c>
       <c r="C84" t="n">
         <v>1</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Channel.C_005</t>
+          <t>Channel.C_002</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>(250.0, 600.0)</t>
+          <t>(100.0, 500.0)</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -3284,11 +3284,11 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>151J</t>
+          <t>110E</t>
         </is>
       </c>
       <c r="H84" t="n">
-        <v>0.73733360090976</v>
+        <v>0.7596852354104493</v>
       </c>
     </row>
     <row r="85">
@@ -3296,19 +3296,19 @@
         <v>83</v>
       </c>
       <c r="B85" s="2" t="n">
-        <v>45230</v>
+        <v>45210</v>
       </c>
       <c r="C85" t="n">
         <v>1</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Channel.C_020</t>
+          <t>Channel.C_002</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>(100.0, 600.0)</t>
+          <t>(100.0, 500.0)</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3318,11 +3318,11 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>7124</t>
+          <t>67G</t>
         </is>
       </c>
       <c r="H85" t="n">
-        <v>0.5774620576220981</v>
+        <v>0.3391859365371409</v>
       </c>
     </row>
     <row r="86">
@@ -3330,19 +3330,19 @@
         <v>84</v>
       </c>
       <c r="B86" s="2" t="n">
-        <v>45230</v>
+        <v>45210</v>
       </c>
       <c r="C86" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Channel.C_020</t>
+          <t>Channel.C_013</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>(100.0, 600.0)</t>
+          <t>(1650.0, 1800.0)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3352,11 +3352,11 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>110E</t>
+          <t>72X</t>
         </is>
       </c>
       <c r="H86" t="n">
-        <v>0.4523922915101564</v>
+        <v>0.2645522633339282</v>
       </c>
     </row>
     <row r="87">
@@ -3364,19 +3364,19 @@
         <v>85</v>
       </c>
       <c r="B87" s="2" t="n">
-        <v>45230</v>
+        <v>45210</v>
       </c>
       <c r="C87" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Channel.C_020</t>
+          <t>Channel.C_002</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>(100.0, 600.0)</t>
+          <t>(0.0, 2000.0)</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -3386,11 +3386,11 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>67G</t>
+          <t>94B</t>
         </is>
       </c>
       <c r="H87" t="n">
-        <v>0.3179354968535256</v>
+        <v>0.8675278958776332</v>
       </c>
     </row>
     <row r="88">
@@ -3398,19 +3398,19 @@
         <v>86</v>
       </c>
       <c r="B88" s="2" t="n">
-        <v>45230</v>
+        <v>45210</v>
       </c>
       <c r="C88" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Channel.C_020</t>
+          <t>Channel.C_002</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>(100.0, 600.0)</t>
+          <t>(0.0, 2000.0)</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -3420,11 +3420,11 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>151J</t>
+          <t>143H</t>
         </is>
       </c>
       <c r="H88" t="n">
-        <v>0.6883589303316482</v>
+        <v>0.2696200995385124</v>
       </c>
     </row>
     <row r="89">
@@ -3432,10 +3432,10 @@
         <v>87</v>
       </c>
       <c r="B89" s="2" t="n">
-        <v>45238</v>
+        <v>45226</v>
       </c>
       <c r="C89" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3444,7 +3444,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>(100.0, 700.0)</t>
+          <t>(1750.0, 1900.0)</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -3454,11 +3454,11 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>7124</t>
+          <t>110E</t>
         </is>
       </c>
       <c r="H89" t="n">
-        <v>0.2843233836190914</v>
+        <v>0.7065371287345135</v>
       </c>
     </row>
     <row r="90">
@@ -3466,19 +3466,19 @@
         <v>88</v>
       </c>
       <c r="B90" s="2" t="n">
-        <v>45238</v>
+        <v>45226</v>
       </c>
       <c r="C90" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Channel.C_007</t>
+          <t>Channel.C_011</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>(100.0, 700.0)</t>
+          <t>(200.0, 700.0)</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -3488,11 +3488,11 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>110E</t>
+          <t>69X</t>
         </is>
       </c>
       <c r="H90" t="n">
-        <v>0.833760761289699</v>
+        <v>0.3430387416450478</v>
       </c>
     </row>
     <row r="91">
@@ -3500,19 +3500,19 @@
         <v>89</v>
       </c>
       <c r="B91" s="2" t="n">
-        <v>45238</v>
+        <v>45226</v>
       </c>
       <c r="C91" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Channel.C_007</t>
+          <t>Channel.C_011</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>(100.0, 700.0)</t>
+          <t>(200.0, 700.0)</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -3522,11 +3522,11 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>67G</t>
+          <t>72X</t>
         </is>
       </c>
       <c r="H91" t="n">
-        <v>0.3273446666980209</v>
+        <v>0.3137935075311603</v>
       </c>
     </row>
     <row r="92">
@@ -3534,32 +3534,1494 @@
         <v>90</v>
       </c>
       <c r="B92" s="2" t="n">
+        <v>45226</v>
+      </c>
+      <c r="C92" t="n">
+        <v>4</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Channel.C_011</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>(200.0, 700.0)</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>143H</t>
+        </is>
+      </c>
+      <c r="H92" t="n">
+        <v>0.363337916347757</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="n">
+        <v>91</v>
+      </c>
+      <c r="B93" s="2" t="n">
+        <v>45226</v>
+      </c>
+      <c r="C93" t="n">
+        <v>4</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Channel.C_020</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>(200.0, 650.0)</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>69X</t>
+        </is>
+      </c>
+      <c r="H93" t="n">
+        <v>0.3961503777414398</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="B94" s="2" t="n">
+        <v>45226</v>
+      </c>
+      <c r="C94" t="n">
+        <v>4</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Channel.C_020</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>(200.0, 650.0)</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>72X</t>
+        </is>
+      </c>
+      <c r="H94" t="n">
+        <v>0.3234602109874793</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="1" t="n">
+        <v>93</v>
+      </c>
+      <c r="B95" s="2" t="n">
+        <v>45226</v>
+      </c>
+      <c r="C95" t="n">
+        <v>4</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Channel.C_020</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>(200.0, 650.0)</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>143H</t>
+        </is>
+      </c>
+      <c r="H95" t="n">
+        <v>0.2972219406496045</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="1" t="n">
+        <v>94</v>
+      </c>
+      <c r="B96" s="2" t="n">
+        <v>45226</v>
+      </c>
+      <c r="C96" t="n">
+        <v>4</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Channel.C_011</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>(0.0, 750.0)</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>72X</t>
+        </is>
+      </c>
+      <c r="H96" t="n">
+        <v>0.2791765997635105</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="1" t="n">
+        <v>95</v>
+      </c>
+      <c r="B97" s="2" t="n">
+        <v>45226</v>
+      </c>
+      <c r="C97" t="n">
+        <v>4</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Channel.C_011</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>(0.0, 750.0)</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>143H</t>
+        </is>
+      </c>
+      <c r="H97" t="n">
+        <v>0.3465263566224303</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="1" t="n">
+        <v>96</v>
+      </c>
+      <c r="B98" s="2" t="n">
+        <v>45226</v>
+      </c>
+      <c r="C98" t="n">
+        <v>4</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Channel.C_011</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>(0.0, 750.0)</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>151J</t>
+        </is>
+      </c>
+      <c r="H98" t="n">
+        <v>0.269613901140984</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="1" t="n">
+        <v>97</v>
+      </c>
+      <c r="B99" s="2" t="n">
+        <v>45226</v>
+      </c>
+      <c r="C99" t="n">
+        <v>4</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Channel.C_020</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>(0.0, 750.0)</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>69X</t>
+        </is>
+      </c>
+      <c r="H99" t="n">
+        <v>0.3052313426782758</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="1" t="n">
+        <v>98</v>
+      </c>
+      <c r="B100" s="2" t="n">
+        <v>45226</v>
+      </c>
+      <c r="C100" t="n">
+        <v>4</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Channel.C_020</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>(0.0, 750.0)</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>72X</t>
+        </is>
+      </c>
+      <c r="H100" t="n">
+        <v>0.3103121198915697</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="1" t="n">
+        <v>99</v>
+      </c>
+      <c r="B101" s="2" t="n">
+        <v>45226</v>
+      </c>
+      <c r="C101" t="n">
+        <v>4</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Channel.C_020</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>(0.0, 750.0)</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>143H</t>
+        </is>
+      </c>
+      <c r="H101" t="n">
+        <v>0.3238740985716736</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B102" s="2" t="n">
+        <v>45250</v>
+      </c>
+      <c r="C102" t="n">
+        <v>1</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Channel.C_013</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>(850.0, 950.0)</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>72X</t>
+        </is>
+      </c>
+      <c r="H102" t="n">
+        <v>0.417942538512428</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="1" t="n">
+        <v>101</v>
+      </c>
+      <c r="B103" s="2" t="n">
+        <v>45250</v>
+      </c>
+      <c r="C103" t="n">
+        <v>1</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Channel.C_013</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>(850.0, 950.0)</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>87J</t>
+        </is>
+      </c>
+      <c r="H103" t="n">
+        <v>0.7461194946627487</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="1" t="n">
+        <v>102</v>
+      </c>
+      <c r="B104" s="2" t="n">
+        <v>45250</v>
+      </c>
+      <c r="C104" t="n">
+        <v>2</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Channel.C_006</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>(2200.0, 2300.0)</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>143H</t>
+        </is>
+      </c>
+      <c r="H104" t="n">
+        <v>0.5744603024202938</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="1" t="n">
+        <v>103</v>
+      </c>
+      <c r="B105" s="2" t="n">
+        <v>45255</v>
+      </c>
+      <c r="C105" t="n">
+        <v>3</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Channel.C_018</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>(50.0, 150.0)</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>7124</t>
+        </is>
+      </c>
+      <c r="H105" t="n">
+        <v>0.5641188924577081</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="1" t="n">
+        <v>104</v>
+      </c>
+      <c r="B106" s="2" t="n">
+        <v>45258</v>
+      </c>
+      <c r="C106" t="n">
+        <v>3</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Channel.C_007</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>(700.0, 850.0)</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>7124</t>
+        </is>
+      </c>
+      <c r="H106" t="n">
+        <v>0.3429585804619826</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="1" t="n">
+        <v>105</v>
+      </c>
+      <c r="B107" s="2" t="n">
+        <v>45258</v>
+      </c>
+      <c r="C107" t="n">
+        <v>4</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Channel.C_015</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>(350.0, 500.0)</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>67G</t>
+        </is>
+      </c>
+      <c r="H107" t="n">
+        <v>0.4491094370986906</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="1" t="n">
+        <v>106</v>
+      </c>
+      <c r="B108" s="2" t="n">
+        <v>45265</v>
+      </c>
+      <c r="C108" t="n">
+        <v>4</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Channel.C_015</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>(650.0, 750.0)</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>72X</t>
+        </is>
+      </c>
+      <c r="H108" t="n">
+        <v>0.3732024309875998</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="1" t="n">
+        <v>107</v>
+      </c>
+      <c r="B109" s="2" t="n">
+        <v>45265</v>
+      </c>
+      <c r="C109" t="n">
+        <v>4</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Channel.C_015</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>(650.0, 750.0)</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>87J</t>
+        </is>
+      </c>
+      <c r="H109" t="n">
+        <v>0.6491349685981751</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="1" t="n">
+        <v>108</v>
+      </c>
+      <c r="B110" s="2" t="n">
+        <v>45274</v>
+      </c>
+      <c r="C110" t="n">
+        <v>1</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Channel.C_024</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>(1450.0, 1750.0)</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>69X</t>
+        </is>
+      </c>
+      <c r="H110" t="n">
+        <v>0.6510734590503868</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="1" t="n">
+        <v>109</v>
+      </c>
+      <c r="B111" s="2" t="n">
+        <v>45274</v>
+      </c>
+      <c r="C111" t="n">
+        <v>1</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Channel.C_024</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>(1450.0, 1750.0)</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>143H</t>
+        </is>
+      </c>
+      <c r="H111" t="n">
+        <v>0.5163293147594377</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="1" t="n">
+        <v>110</v>
+      </c>
+      <c r="B112" s="2" t="n">
+        <v>45274</v>
+      </c>
+      <c r="C112" t="n">
+        <v>1</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Channel.C_024</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>(1450.0, 1750.0)</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>151J</t>
+        </is>
+      </c>
+      <c r="H112" t="n">
+        <v>0.2814813738336527</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="1" t="n">
+        <v>111</v>
+      </c>
+      <c r="B113" s="2" t="n">
+        <v>45274</v>
+      </c>
+      <c r="C113" t="n">
+        <v>4</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Channel.C_006</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>(1900.0, 2000.0)</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>7124</t>
+        </is>
+      </c>
+      <c r="H113" t="n">
+        <v>0.6381071099002988</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="1" t="n">
+        <v>112</v>
+      </c>
+      <c r="B114" s="2" t="n">
+        <v>45274</v>
+      </c>
+      <c r="C114" t="n">
+        <v>4</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Channel.C_006</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>(1900.0, 2000.0)</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>151J</t>
+        </is>
+      </c>
+      <c r="H114" t="n">
+        <v>0.2895380481587378</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="1" t="n">
+        <v>113</v>
+      </c>
+      <c r="B115" s="2" t="n">
+        <v>45274</v>
+      </c>
+      <c r="C115" t="n">
+        <v>4</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Channel.C_008</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>(750.0, 850.0)</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>7124</t>
+        </is>
+      </c>
+      <c r="H115" t="n">
+        <v>0.6756920806691046</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="1" t="n">
+        <v>114</v>
+      </c>
+      <c r="B116" s="2" t="n">
+        <v>45274</v>
+      </c>
+      <c r="C116" t="n">
+        <v>4</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Channel.C_008</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>(750.0, 850.0)</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>151J</t>
+        </is>
+      </c>
+      <c r="H116" t="n">
+        <v>0.6501479915433404</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="1" t="n">
+        <v>115</v>
+      </c>
+      <c r="B117" s="2" t="n">
+        <v>45278</v>
+      </c>
+      <c r="C117" t="n">
+        <v>2</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Channel.C_012_Unit 2</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>(200.0, 350.0)</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>72X</t>
+        </is>
+      </c>
+      <c r="H117" t="n">
+        <v>0.5614544939041679</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="1" t="n">
+        <v>116</v>
+      </c>
+      <c r="B118" s="2" t="n">
+        <v>45278</v>
+      </c>
+      <c r="C118" t="n">
+        <v>2</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Channel.C_012_Unit 2</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>(200.0, 350.0)</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>87J</t>
+        </is>
+      </c>
+      <c r="H118" t="n">
+        <v>0.6856713552318544</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="1" t="n">
+        <v>117</v>
+      </c>
+      <c r="B119" s="2" t="n">
+        <v>45278</v>
+      </c>
+      <c r="C119" t="n">
+        <v>3</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Channel.C_020_Unit 1</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>(150.0, 400.0)</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>87J</t>
+        </is>
+      </c>
+      <c r="H119" t="n">
+        <v>0.7393426952957101</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="1" t="n">
+        <v>118</v>
+      </c>
+      <c r="B120" s="2" t="n">
+        <v>45195</v>
+      </c>
+      <c r="C120" t="n">
+        <v>1</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Channel.C_027_Unit 1</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>(0.0, 300.0)</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>94B</t>
+        </is>
+      </c>
+      <c r="H120" t="n">
+        <v>0.5817645073627393</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="1" t="n">
+        <v>119</v>
+      </c>
+      <c r="B121" s="2" t="n">
+        <v>45223</v>
+      </c>
+      <c r="C121" t="n">
+        <v>2</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Channel.C_002</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>(250.0, 750.0)</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>94B</t>
+        </is>
+      </c>
+      <c r="H121" t="n">
+        <v>0.7461224024765438</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="1" t="n">
+        <v>120</v>
+      </c>
+      <c r="B122" s="2" t="n">
+        <v>45223</v>
+      </c>
+      <c r="C122" t="n">
+        <v>2</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Channel.C_002</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>(250.0, 750.0)</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>143H</t>
+        </is>
+      </c>
+      <c r="H122" t="n">
+        <v>0.261013043787052</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="1" t="n">
+        <v>121</v>
+      </c>
+      <c r="B123" s="2" t="n">
+        <v>45223</v>
+      </c>
+      <c r="C123" t="n">
+        <v>2</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Channel.C_002</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>(250.0, 750.0)</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>151J</t>
+        </is>
+      </c>
+      <c r="H123" t="n">
+        <v>0.4522559139679887</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="1" t="n">
+        <v>122</v>
+      </c>
+      <c r="B124" s="2" t="n">
+        <v>45230</v>
+      </c>
+      <c r="C124" t="n">
+        <v>1</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Channel.C_005</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>(250.0, 600.0)</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>7124</t>
+        </is>
+      </c>
+      <c r="H124" t="n">
+        <v>0.4626862340052377</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="1" t="n">
+        <v>123</v>
+      </c>
+      <c r="B125" s="2" t="n">
+        <v>45230</v>
+      </c>
+      <c r="C125" t="n">
+        <v>1</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Channel.C_005</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>(250.0, 600.0)</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>143H</t>
+        </is>
+      </c>
+      <c r="H125" t="n">
+        <v>0.2784554922691393</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="1" t="n">
+        <v>124</v>
+      </c>
+      <c r="B126" s="2" t="n">
+        <v>45230</v>
+      </c>
+      <c r="C126" t="n">
+        <v>1</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Channel.C_005</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>(250.0, 600.0)</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>87J</t>
+        </is>
+      </c>
+      <c r="H126" t="n">
+        <v>0.3519294547137312</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="1" t="n">
+        <v>125</v>
+      </c>
+      <c r="B127" s="2" t="n">
+        <v>45230</v>
+      </c>
+      <c r="C127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Channel.C_005</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>(250.0, 600.0)</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>151J</t>
+        </is>
+      </c>
+      <c r="H127" t="n">
+        <v>0.73733360090976</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="1" t="n">
+        <v>126</v>
+      </c>
+      <c r="B128" s="2" t="n">
+        <v>45230</v>
+      </c>
+      <c r="C128" t="n">
+        <v>1</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Channel.C_020</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>(100.0, 600.0)</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>7124</t>
+        </is>
+      </c>
+      <c r="H128" t="n">
+        <v>0.5774620576220981</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="1" t="n">
+        <v>127</v>
+      </c>
+      <c r="B129" s="2" t="n">
+        <v>45230</v>
+      </c>
+      <c r="C129" t="n">
+        <v>1</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Channel.C_020</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>(100.0, 600.0)</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>110E</t>
+        </is>
+      </c>
+      <c r="H129" t="n">
+        <v>0.4523922915101564</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="1" t="n">
+        <v>128</v>
+      </c>
+      <c r="B130" s="2" t="n">
+        <v>45230</v>
+      </c>
+      <c r="C130" t="n">
+        <v>1</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Channel.C_020</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>(100.0, 600.0)</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>67G</t>
+        </is>
+      </c>
+      <c r="H130" t="n">
+        <v>0.3179354968535256</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="1" t="n">
+        <v>129</v>
+      </c>
+      <c r="B131" s="2" t="n">
+        <v>45230</v>
+      </c>
+      <c r="C131" t="n">
+        <v>1</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Channel.C_020</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>(100.0, 600.0)</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>151J</t>
+        </is>
+      </c>
+      <c r="H131" t="n">
+        <v>0.6883589303316482</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="1" t="n">
+        <v>130</v>
+      </c>
+      <c r="B132" s="2" t="n">
         <v>45238</v>
       </c>
-      <c r="C92" t="n">
+      <c r="C132" t="n">
         <v>1</v>
       </c>
-      <c r="D92" t="inlineStr">
+      <c r="D132" t="inlineStr">
         <is>
           <t>Channel.C_007</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr">
+      <c r="E132" t="inlineStr">
         <is>
           <t>(100.0, 700.0)</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>AffliationFrom</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>7124</t>
+        </is>
+      </c>
+      <c r="H132" t="n">
+        <v>0.2843233836190914</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="1" t="n">
+        <v>131</v>
+      </c>
+      <c r="B133" s="2" t="n">
+        <v>45238</v>
+      </c>
+      <c r="C133" t="n">
+        <v>1</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Channel.C_007</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>(100.0, 700.0)</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>110E</t>
+        </is>
+      </c>
+      <c r="H133" t="n">
+        <v>0.833760761289699</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="1" t="n">
+        <v>132</v>
+      </c>
+      <c r="B134" s="2" t="n">
+        <v>45238</v>
+      </c>
+      <c r="C134" t="n">
+        <v>1</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Channel.C_007</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>(100.0, 700.0)</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>67G</t>
+        </is>
+      </c>
+      <c r="H134" t="n">
+        <v>0.3273446666980209</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="1" t="n">
+        <v>133</v>
+      </c>
+      <c r="B135" s="2" t="n">
+        <v>45238</v>
+      </c>
+      <c r="C135" t="n">
+        <v>1</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Channel.C_007</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>(100.0, 700.0)</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>AffliationFrom</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
         <is>
           <t>151J</t>
         </is>
       </c>
-      <c r="H92" t="n">
+      <c r="H135" t="n">
         <v>0.3975313700384123</v>
       </c>
     </row>

</xml_diff>